<commit_message>
Added multiple code columns to code config file. Execute code in order until we get a non-empty value.
</commit_message>
<xml_diff>
--- a/data/odm_v2/odm_v2_id_code.xlsx
+++ b/data/odm_v2/odm_v2_id_code.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-MapGenerator/PHES-ODM-MapGenerator/data/odm_v2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA7E8D09-53E7-DE4A-B21A-5B6498E778C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D64BC489-1F4E-C54E-A2B1-1A19E5E49DE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20940" xr2:uid="{0C2D13F0-D956-9E49-BD3E-392F28BA92F9}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="77">
   <si>
     <t>addresses</t>
   </si>
@@ -160,9 +160,6 @@
     <t>zones</t>
   </si>
   <si>
-    <t>code</t>
-  </si>
-  <si>
     <t>dat.addresses.addressID</t>
   </si>
   <si>
@@ -245,6 +242,30 @@
   </si>
   <si>
     <t>dat.measureSets.measureSetRepID if dat0.qualityReports.__measureSetRepID else ""</t>
+  </si>
+  <si>
+    <t>code0</t>
+  </si>
+  <si>
+    <t>dat0.contacts.__contactID</t>
+  </si>
+  <si>
+    <t>dat0.organizations.__organizationID</t>
+  </si>
+  <si>
+    <t>dat0.samples.__sampleID</t>
+  </si>
+  <si>
+    <t>dat0.protocols.__protocolID</t>
+  </si>
+  <si>
+    <t>dat0.sites.__siteID</t>
+  </si>
+  <si>
+    <t>dat0.datasets.__datasetID</t>
+  </si>
+  <si>
+    <t>code1</t>
   </si>
 </sst>
 </file>
@@ -268,18 +289,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.14999847407452621"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -296,8 +311,8 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -612,44 +627,50 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3A1991E-0020-B448-B50F-72C1AC9C88C8}">
-  <dimension ref="A1:D88"/>
+  <dimension ref="A1:E88"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="15.83203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="113" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.83203125" style="2"/>
+    <col min="2" max="2" width="15.83203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="81.6640625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="113" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="10.83203125" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>59</v>
-      </c>
       <c r="C1" s="1" t="s">
-        <v>41</v>
+        <v>69</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C2" t="s">
-        <v>63</v>
+      <c r="C2" s="2" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+      <c r="A3" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C3" t="s">
-        <v>43</v>
+      <c r="C3" s="2" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
@@ -660,7 +681,10 @@
         <v>11</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>54</v>
+        <v>70</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
@@ -671,7 +695,7 @@
         <v>2</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
@@ -682,15 +706,13 @@
         <v>10</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
@@ -699,7 +721,6 @@
       <c r="B11" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="2"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
@@ -708,9 +729,11 @@
       <c r="B12" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C12" s="2"/>
+      <c r="C12" s="2" t="s">
+        <v>75</v>
+      </c>
       <c r="D12" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
@@ -720,7 +743,6 @@
       <c r="B13" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C13" s="2"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
@@ -729,7 +751,6 @@
       <c r="B14" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C14" s="2"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
@@ -738,7 +759,6 @@
       <c r="B15" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C15" s="2"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
@@ -747,7 +767,6 @@
       <c r="B16" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C16" s="2"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
@@ -757,7 +776,7 @@
         <v>16</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
@@ -768,7 +787,7 @@
         <v>2</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
@@ -779,7 +798,7 @@
         <v>11</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
@@ -790,113 +809,111 @@
         <v>10</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
+      <c r="A25" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C25" t="s">
-        <v>64</v>
+      <c r="C25" s="2" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
+      <c r="A26" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C26" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A27" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C27" s="2" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A28" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B27" t="s">
-        <v>6</v>
-      </c>
-      <c r="C27" t="s">
+      <c r="B28" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A29" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C29" s="2" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A28" t="s">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A30" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B28" t="s">
-        <v>7</v>
-      </c>
-      <c r="C28" t="s">
+      <c r="B30" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A31" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C31" s="2" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A29" t="s">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A32" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B29" t="s">
-        <v>8</v>
-      </c>
-      <c r="C29" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A30" t="s">
+      <c r="B32" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A33" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B30" t="s">
-        <v>2</v>
-      </c>
-      <c r="C30" t="s">
+      <c r="B33" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C33" s="2" t="s">
         <v>43</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A31" t="s">
-        <v>3</v>
-      </c>
-      <c r="B31" t="s">
-        <v>9</v>
-      </c>
-      <c r="C31" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A32" t="s">
-        <v>3</v>
-      </c>
-      <c r="B32" t="s">
-        <v>10</v>
-      </c>
-      <c r="C32" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A33" t="s">
-        <v>3</v>
-      </c>
-      <c r="B33" t="s">
-        <v>11</v>
-      </c>
-      <c r="C33" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
@@ -907,7 +924,7 @@
         <v>9</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
@@ -918,7 +935,7 @@
         <v>5</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
@@ -929,7 +946,7 @@
         <v>10</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
@@ -940,7 +957,7 @@
         <v>11</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
@@ -950,9 +967,11 @@
       <c r="B40" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C40" s="2"/>
+      <c r="C40" s="2" t="s">
+        <v>71</v>
+      </c>
       <c r="D40" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
@@ -963,7 +982,7 @@
         <v>1</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
@@ -974,7 +993,7 @@
         <v>2</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
@@ -985,7 +1004,7 @@
         <v>7</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
@@ -996,7 +1015,7 @@
         <v>2</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
@@ -1007,7 +1026,7 @@
         <v>10</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
@@ -1018,319 +1037,324 @@
         <v>11</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B49" s="2"/>
-      <c r="C49" s="2"/>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A51" t="s">
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A51" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B51" t="s">
+      <c r="B51" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A52" t="s">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A52" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B52" t="s">
+      <c r="B52" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D52" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A53" t="s">
+      <c r="C52" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A53" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B53" t="s">
+      <c r="B53" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C53" t="s">
+      <c r="C53" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A54" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A55" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C55" s="2" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A54" t="s">
-        <v>12</v>
-      </c>
-      <c r="B54" t="s">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A57" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E57" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A58" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B58" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C54" t="s">
+      <c r="C58" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A59" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A60" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C60" s="2" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A55" t="s">
-        <v>12</v>
-      </c>
-      <c r="B55" t="s">
-        <v>11</v>
-      </c>
-      <c r="C55" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A57" t="s">
-        <v>14</v>
-      </c>
-      <c r="B57" t="s">
-        <v>15</v>
-      </c>
-      <c r="C57" t="s">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A62" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A63" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A64" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C64" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="D57" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A58" t="s">
-        <v>14</v>
-      </c>
-      <c r="B58" t="s">
-        <v>10</v>
-      </c>
-      <c r="C58" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A59" t="s">
-        <v>14</v>
-      </c>
-      <c r="B59" t="s">
-        <v>11</v>
-      </c>
-      <c r="C59" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A60" t="s">
-        <v>14</v>
-      </c>
-      <c r="B60" t="s">
-        <v>16</v>
-      </c>
-      <c r="C60" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A62" t="s">
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A65" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B62" t="s">
-        <v>18</v>
-      </c>
-      <c r="C62" t="s">
+      <c r="B65" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C65" s="2" t="s">
         <v>68</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A63" t="s">
-        <v>17</v>
-      </c>
-      <c r="B63" t="s">
-        <v>4</v>
-      </c>
-      <c r="C63" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A64" t="s">
-        <v>17</v>
-      </c>
-      <c r="B64" t="s">
-        <v>6</v>
-      </c>
-      <c r="C64" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A65" t="s">
-        <v>17</v>
-      </c>
-      <c r="B65" t="s">
-        <v>9</v>
-      </c>
-      <c r="C65" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A67" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B67" s="2"/>
-      <c r="C67" s="2"/>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A69" t="s">
+      <c r="A69" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B69" t="s">
+      <c r="B69" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D69" t="s">
-        <v>61</v>
+      <c r="C69" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D69" s="2" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A70" t="s">
+      <c r="A70" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B70" t="s">
+      <c r="B70" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C70" t="s">
-        <v>45</v>
+      <c r="C70" s="2" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A71" t="s">
+      <c r="A71" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B71" t="s">
+      <c r="B71" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C71" t="s">
-        <v>50</v>
+      <c r="C71" s="2" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A72" t="s">
+      <c r="A72" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B72" t="s">
+      <c r="B72" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C72" t="s">
-        <v>44</v>
+      <c r="C72" s="2" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A73" t="s">
+      <c r="A73" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B73" t="s">
+      <c r="B73" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C73" t="s">
+      <c r="C73" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A74" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A76" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A77" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D77" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A78" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A79" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C79" s="2" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A74" t="s">
-        <v>19</v>
-      </c>
-      <c r="B74" t="s">
-        <v>2</v>
-      </c>
-      <c r="C74" t="s">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A80" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C80" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A81" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C81" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A82" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C82" s="2" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A76" t="s">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A83" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B76" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A77" t="s">
+      <c r="B83" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A84" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B77" t="s">
-        <v>8</v>
-      </c>
-      <c r="C77" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A78" t="s">
-        <v>20</v>
-      </c>
-      <c r="B78" t="s">
-        <v>2</v>
-      </c>
-      <c r="C78" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A79" t="s">
-        <v>20</v>
-      </c>
-      <c r="B79" t="s">
-        <v>7</v>
-      </c>
-      <c r="C79" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A80" t="s">
-        <v>20</v>
-      </c>
-      <c r="B80" t="s">
-        <v>1</v>
-      </c>
-      <c r="C80" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A81" t="s">
-        <v>20</v>
-      </c>
-      <c r="B81" t="s">
-        <v>10</v>
-      </c>
-      <c r="C81" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A82" t="s">
-        <v>20</v>
-      </c>
-      <c r="B82" t="s">
-        <v>11</v>
-      </c>
-      <c r="C82" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A83" t="s">
-        <v>20</v>
-      </c>
-      <c r="B83" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A84" t="s">
-        <v>20</v>
-      </c>
-      <c r="B84" t="s">
+      <c r="B84" s="2" t="s">
         <v>23</v>
       </c>
     </row>
@@ -1338,15 +1362,11 @@
       <c r="A86" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B86" s="2"/>
-      <c r="C86" s="2"/>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A88" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B88" s="2"/>
-      <c r="C88" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Updates to ID generation code
</commit_message>
<xml_diff>
--- a/data/odm_v2/odm_v2_id_code.xlsx
+++ b/data/odm_v2/odm_v2_id_code.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-MapGenerator/PHES-ODM-MapGenerator/data/odm_v2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2E07A31-FB41-1448-AB62-792AA117F973}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30E1AFF4-930E-5445-95A4-8A3E0AE7FB56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20920" xr2:uid="{0C2D13F0-D956-9E49-BD3E-392F28BA92F9}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="86">
   <si>
     <t>addresses</t>
   </si>
@@ -160,115 +160,139 @@
     <t>zones</t>
   </si>
   <si>
+    <t>class</t>
+  </si>
+  <si>
+    <t>slot</t>
+  </si>
+  <si>
+    <t>code0</t>
+  </si>
+  <si>
+    <t>code1</t>
+  </si>
+  <si>
+    <t>fn.makeid(datEmpty.qualityReports.qualityFlag, datEmpty.qualityReports.measureRepID if datEmpty.qualityReports.__measureRepID else datEmpty.qualityReports.sampleID if datEmpty.qualityReports.__sampleID else datEmpty.qualityReports.measureSetRepID)</t>
+  </si>
+  <si>
+    <t>dat.addresses.__addressID</t>
+  </si>
+  <si>
+    <t>dat.datasets.datasetID</t>
+  </si>
+  <si>
+    <t>dat.contacts.__contactID</t>
+  </si>
+  <si>
+    <t>dat.organizations.organizationID</t>
+  </si>
+  <si>
+    <t>dat.datasets.__datasetID</t>
+  </si>
+  <si>
+    <t>dat.instruments.__instrumentID</t>
+  </si>
+  <si>
+    <t>dat.contacts.contactID</t>
+  </si>
+  <si>
+    <t>dat.measures.__measureRepID</t>
+  </si>
+  <si>
+    <t>dat.protocols.protocolID</t>
+  </si>
+  <si>
+    <t>dat.samples.sampleID</t>
+  </si>
+  <si>
+    <t>dat.polygons.polygonID</t>
+  </si>
+  <si>
+    <t>dat.sites.siteID</t>
+  </si>
+  <si>
+    <t>dat.measureSets.measureSetRepID</t>
+  </si>
+  <si>
+    <t>dat.organizations.__organizationID</t>
+  </si>
+  <si>
     <t>dat.addresses.addressID</t>
   </si>
   <si>
-    <t>dat.datasets.datasetID</t>
-  </si>
-  <si>
-    <t>dat.contacts.contactID</t>
-  </si>
-  <si>
-    <t>dat.protocols.protocolID</t>
-  </si>
-  <si>
-    <t>dat.samples.sampleID</t>
-  </si>
-  <si>
-    <t>dat.sites.siteID</t>
-  </si>
-  <si>
-    <t>dat.polygons.polygonID</t>
-  </si>
-  <si>
-    <t>dat.measureSets.measureSetRepID</t>
-  </si>
-  <si>
-    <t>dat.organizations.organizationID</t>
+    <t>dat.polygons.__polygonID</t>
+  </si>
+  <si>
+    <t>dat.protocols.__protocolID</t>
+  </si>
+  <si>
+    <t>dat.protocolSteps.__stepID</t>
   </si>
   <si>
     <t>dat.instruments.instrumentID</t>
   </si>
   <si>
-    <t>fn.makeid(dat.protocols.name, dat.protocols.protocolVersion)</t>
-  </si>
-  <si>
-    <t>fn.makeid(dat.addresses.country, dat.addresses.pCode, dat.addresses.city[:3], dat.sites.name[:3])</t>
-  </si>
-  <si>
-    <t>fn.makeid(dat.organizations.organizationID, dat.contacts.role[:3])</t>
-  </si>
-  <si>
-    <t>fn.makeid(dat.organizations.organizationID, dat.sites.siteID)</t>
-  </si>
-  <si>
-    <t>class</t>
-  </si>
-  <si>
-    <t>slot</t>
-  </si>
-  <si>
-    <t>fn.makeid(dat.samples.siteID, fn.date(dat.samples.collDT) if dat.samples.collDT else fn.date(dat.samples.collDTEnd), fn.rownum)</t>
-  </si>
-  <si>
-    <t>fn.makeid(dat.instruments.manufacturer, dat.instruments.name[:3], dat.instruments.model[:3], fn.rownum)</t>
-  </si>
-  <si>
-    <t>fn.makeid(dat.addresses.country, dat.addresses.pCode, dat.addresses.city[:3], fn.rownum)</t>
-  </si>
-  <si>
-    <t>fn.makeid(dat.measures.sampleID, dat.measures.measure, fn.rownum)</t>
-  </si>
-  <si>
-    <t>fn.makeid(dat.organizations.organizationID, dat.protocolSteps.measure[-3:] if dat0.protocolSteps.measure else dat.protocolSteps.method[-3:])</t>
-  </si>
-  <si>
-    <t>dat.samples.sampleID if dat0.qualityReports.__sampleID else ""</t>
-  </si>
-  <si>
-    <t>dat.measures.measureRepID if dat0.qualityReports.__measureRepID else ""</t>
-  </si>
-  <si>
-    <t>fn.makeid(dat.qualityReports.qualityFlag, dat.qualityReports.measureRepID if dat0.qualityReports.__measureRepID else dat.qualityReports.sampleID if dat0.qualityReports.__sampleID else dat.qualityReports.measureSetRepID)</t>
-  </si>
-  <si>
-    <t>dat.measureSets.measureSetRepID if dat0.qualityReports.__measureSetRepID else ""</t>
-  </si>
-  <si>
-    <t>code0</t>
-  </si>
-  <si>
-    <t>dat0.contacts.__contactID</t>
-  </si>
-  <si>
-    <t>dat0.organizations.__organizationID</t>
-  </si>
-  <si>
-    <t>dat0.samples.__sampleID</t>
-  </si>
-  <si>
-    <t>dat0.protocols.__protocolID</t>
-  </si>
-  <si>
-    <t>dat0.sites.__siteID</t>
-  </si>
-  <si>
-    <t>dat0.datasets.__datasetID</t>
-  </si>
-  <si>
-    <t>code1</t>
-  </si>
-  <si>
-    <t>fn.makeid(dat.measures.measureRepID, "{:04d}".format(fn.countrows("measures", "__measureSetRepID", equals=dat.measureSets.__measureSetRepID)))</t>
-  </si>
-  <si>
-    <t>fn.makeid(dat.addresses.addressID, dat.organizations.name[:3])</t>
-  </si>
-  <si>
-    <t>fn.makeid(dat.addresses.country, dat.addresses.pCode, dat.addresses.city[:3])</t>
-  </si>
-  <si>
-    <t>fn.makeid(dat.instruments.manufacturer, dat.instruments.name[:3], dat.instruments.model[:3])</t>
+    <t>dat.measures.measureRepID if dat.qualityReports.__measureRepID else ""</t>
+  </si>
+  <si>
+    <t>dat.samples.sampleID if dat.qualityReports.__sampleID else ""</t>
+  </si>
+  <si>
+    <t>dat.measureSets.measureSetRepID if dat.qualityReports.__measureSetRepID else ""</t>
+  </si>
+  <si>
+    <t>dat.samples.__sampleID</t>
+  </si>
+  <si>
+    <t>dat.sites.__siteID</t>
+  </si>
+  <si>
+    <t>fn.makeid(datEmpty.addresses.country, datEmpty.addresses.pCode, datEmpty.addresses.city[:3])</t>
+  </si>
+  <si>
+    <t>fn.makeid(datEmpty.addresses.country, datEmpty.addresses.pCode, datEmpty.addresses.city[:3], fn.rownum)</t>
+  </si>
+  <si>
+    <t>fn.makeid(datEmpty.organizations.organizationID, datEmpty.contacts.role[:3])</t>
+  </si>
+  <si>
+    <t>fn.makeid(datEmpty.instruments.manufacturer, datEmpty.instruments.name[:3], datEmpty.instruments.model[:3])</t>
+  </si>
+  <si>
+    <t>fn.makeid(datEmpty.instruments.manufacturer, datEmpty.instruments.name[:3], datEmpty.instruments.model[:3], fn.rownum)</t>
+  </si>
+  <si>
+    <t>fn.makeid(datEmpty.measures.sampleID, datEmpty.measures.measure)</t>
+  </si>
+  <si>
+    <t>fn.makeid(datEmpty.measures.sampleID, datEmpty.measures.measure, fn.rownum)</t>
+  </si>
+  <si>
+    <t>fn.makeid(datEmpty.measures.measureRepID, "{:04d}".format(fn.countrows("measures", "__measureSetRepID", equals=datEmpty.measureSets.__measureSetRepID)))</t>
+  </si>
+  <si>
+    <t>fn.makeid(datEmpty.addresses.addressID, datEmpty.organizations.name[:3])</t>
+  </si>
+  <si>
+    <t>fn.makeid(datEmpty.organizations.organizationID, datEmpty.sites.siteID)</t>
+  </si>
+  <si>
+    <t>fn.makeid(datEmpty.protocols.name, datEmpty.protocols.protocolVersion)</t>
+  </si>
+  <si>
+    <t>fn.makeid(datEmpty.organizations.organizationID, datEmpty.protocolSteps.measure[-3:] if datEmpty.protocolSteps.measure else datEmpty.protocolSteps.method[-3:])</t>
+  </si>
+  <si>
+    <t>datEmpty.qualityReports.__qualityReportID</t>
+  </si>
+  <si>
+    <t>fn.makeid(datEmpty.samples.siteID, fn.date(datEmpty.samples.collDT) if datEmpty.samples.collDT else fn.date(datEmpty.samples.collDTEnd), fn.rownum)</t>
+  </si>
+  <si>
+    <t>fn.makeid(datEmpty.addresses.country, datEmpty.addresses.pCode, datEmpty.addresses.city[:3], datEmpty.sites.name[:3])</t>
+  </si>
+  <si>
+    <t>fn.makeid(datEmpty.measures.measureRepID, "{:04d}".format(fn.countrows("measures", "__measureSetRepID", equals=dat.measureSets.__measureSetRepID)))</t>
   </si>
 </sst>
 </file>
@@ -640,16 +664,16 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>55</v>
+        <v>41</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>56</v>
+        <v>42</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>66</v>
+        <v>43</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>73</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
@@ -660,10 +684,13 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>76</v>
+        <v>46</v>
+      </c>
+      <c r="D2" t="s">
+        <v>70</v>
       </c>
       <c r="E2" t="s">
-        <v>59</v>
+        <v>71</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -674,7 +701,7 @@
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
@@ -685,10 +712,10 @@
         <v>11</v>
       </c>
       <c r="C5" t="s">
-        <v>67</v>
+        <v>48</v>
       </c>
       <c r="D5" t="s">
-        <v>53</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
@@ -699,7 +726,7 @@
         <v>2</v>
       </c>
       <c r="C6" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
@@ -734,7 +761,7 @@
         <v>2</v>
       </c>
       <c r="C12" t="s">
-        <v>72</v>
+        <v>50</v>
       </c>
       <c r="D12" t="s">
         <v>49</v>
@@ -780,10 +807,13 @@
         <v>16</v>
       </c>
       <c r="C18" t="s">
-        <v>77</v>
+        <v>51</v>
+      </c>
+      <c r="D18" t="s">
+        <v>73</v>
       </c>
       <c r="E18" t="s">
-        <v>58</v>
+        <v>74</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
@@ -794,7 +824,7 @@
         <v>2</v>
       </c>
       <c r="C19" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
@@ -805,7 +835,7 @@
         <v>11</v>
       </c>
       <c r="C20" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
@@ -832,10 +862,13 @@
         <v>4</v>
       </c>
       <c r="C25" t="s">
-        <v>60</v>
+        <v>53</v>
+      </c>
+      <c r="D25" t="s">
+        <v>75</v>
       </c>
       <c r="E25" t="s">
-        <v>60</v>
+        <v>76</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
@@ -846,7 +879,7 @@
         <v>5</v>
       </c>
       <c r="C26" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
@@ -857,7 +890,7 @@
         <v>6</v>
       </c>
       <c r="C27" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
@@ -868,7 +901,7 @@
         <v>7</v>
       </c>
       <c r="C28" t="s">
-        <v>47</v>
+        <v>56</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
@@ -879,7 +912,7 @@
         <v>8</v>
       </c>
       <c r="C29" t="s">
-        <v>46</v>
+        <v>57</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
@@ -890,7 +923,7 @@
         <v>2</v>
       </c>
       <c r="C30" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
@@ -901,7 +934,7 @@
         <v>9</v>
       </c>
       <c r="C31" t="s">
-        <v>48</v>
+        <v>58</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
@@ -915,7 +948,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>3</v>
       </c>
@@ -923,10 +956,10 @@
         <v>11</v>
       </c>
       <c r="C33" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>34</v>
       </c>
@@ -934,10 +967,13 @@
         <v>9</v>
       </c>
       <c r="C35" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
+        <v>85</v>
+      </c>
+      <c r="E35" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>34</v>
       </c>
@@ -945,10 +981,10 @@
         <v>5</v>
       </c>
       <c r="C36" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>34</v>
       </c>
@@ -959,7 +995,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>34</v>
       </c>
@@ -967,10 +1003,10 @@
         <v>11</v>
       </c>
       <c r="C38" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>35</v>
       </c>
@@ -978,13 +1014,13 @@
         <v>10</v>
       </c>
       <c r="C40" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="D40" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>35</v>
       </c>
@@ -992,10 +1028,10 @@
         <v>1</v>
       </c>
       <c r="C41" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>35</v>
       </c>
@@ -1003,10 +1039,10 @@
         <v>2</v>
       </c>
       <c r="C42" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>36</v>
       </c>
@@ -1014,10 +1050,13 @@
         <v>7</v>
       </c>
       <c r="C44" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
+        <v>61</v>
+      </c>
+      <c r="D44" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>36</v>
       </c>
@@ -1025,10 +1064,10 @@
         <v>2</v>
       </c>
       <c r="C45" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>36</v>
       </c>
@@ -1039,7 +1078,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>36</v>
       </c>
@@ -1047,7 +1086,7 @@
         <v>11</v>
       </c>
       <c r="C47" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
@@ -1071,10 +1110,10 @@
         <v>5</v>
       </c>
       <c r="C52" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="D52" t="s">
-        <v>51</v>
+        <v>80</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.2">
@@ -1085,7 +1124,7 @@
         <v>2</v>
       </c>
       <c r="C53" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.2">
@@ -1107,7 +1146,7 @@
         <v>11</v>
       </c>
       <c r="C55" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.2">
@@ -1118,7 +1157,10 @@
         <v>15</v>
       </c>
       <c r="C57" t="s">
-        <v>61</v>
+        <v>63</v>
+      </c>
+      <c r="D57" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.2">
@@ -1140,7 +1182,7 @@
         <v>11</v>
       </c>
       <c r="C59" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.2">
@@ -1151,7 +1193,7 @@
         <v>16</v>
       </c>
       <c r="C60" t="s">
-        <v>50</v>
+        <v>64</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.2">
@@ -1162,7 +1204,10 @@
         <v>18</v>
       </c>
       <c r="C62" t="s">
-        <v>64</v>
+        <v>82</v>
+      </c>
+      <c r="D62" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.2">
@@ -1173,7 +1218,7 @@
         <v>4</v>
       </c>
       <c r="C63" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.2">
@@ -1184,7 +1229,7 @@
         <v>6</v>
       </c>
       <c r="C64" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.2">
@@ -1195,7 +1240,7 @@
         <v>9</v>
       </c>
       <c r="C65" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.2">
@@ -1211,10 +1256,10 @@
         <v>6</v>
       </c>
       <c r="C69" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D69" t="s">
-        <v>57</v>
+        <v>83</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.2">
@@ -1225,7 +1270,7 @@
         <v>5</v>
       </c>
       <c r="C70" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.2">
@@ -1247,7 +1292,7 @@
         <v>11</v>
       </c>
       <c r="C72" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.2">
@@ -1258,7 +1303,7 @@
         <v>8</v>
       </c>
       <c r="C73" t="s">
-        <v>46</v>
+        <v>57</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.2">
@@ -1269,7 +1314,7 @@
         <v>2</v>
       </c>
       <c r="C74" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.2">
@@ -1288,10 +1333,10 @@
         <v>8</v>
       </c>
       <c r="C77" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D77" t="s">
-        <v>52</v>
+        <v>84</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.2">
@@ -1302,7 +1347,7 @@
         <v>2</v>
       </c>
       <c r="C78" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.2">
@@ -1313,7 +1358,7 @@
         <v>7</v>
       </c>
       <c r="C79" t="s">
-        <v>47</v>
+        <v>56</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.2">
@@ -1324,7 +1369,7 @@
         <v>1</v>
       </c>
       <c r="C80" t="s">
-        <v>41</v>
+        <v>60</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.2">
@@ -1346,7 +1391,7 @@
         <v>11</v>
       </c>
       <c r="C82" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.2">

</xml_diff>